<commit_message>
some changes and add category
</commit_message>
<xml_diff>
--- a/data/images.xlsx
+++ b/data/images.xlsx
@@ -4,6 +4,7 @@
   <workbookPr codeName="ThisWorkbook"/>
   <sheets>
     <sheet name="Images" sheetId="1" r:id="rId1"/>
+    <sheet name="Categories" sheetId="2" r:id="rId2"/>
   </sheets>
 </workbook>
 </file>
@@ -397,333 +398,43 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:D23"/>
+  <dimension ref="A1"/>
+  <sheetData/>
+  <ignoredErrors>
+    <ignoredError numberStoredAsText="1" sqref="A1"/>
+  </ignoredErrors>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
+  <dimension ref="A1:C2"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
         <v>id</v>
       </c>
       <c r="B1" t="str">
-        <v>label</v>
+        <v>name</v>
       </c>
       <c r="C1" t="str">
-        <v>url</v>
-      </c>
-      <c r="D1" t="str">
         <v>createdAt</v>
       </c>
     </row>
     <row r="2">
       <c r="A2" t="str">
-        <v>img-001</v>
+        <v>cat-001</v>
       </c>
       <c r="B2" t="str">
-        <v>Pexels Dog</v>
+        <v>عام</v>
       </c>
       <c r="C2" t="str">
-        <v>https://images.pexels.com/photos/802112/pexels-photo-802112.jpeg</v>
-      </c>
-      <c r="D2" t="str">
-        <v>2026-02-21T00:04:56.454Z</v>
-      </c>
-    </row>
-    <row r="3">
-      <c r="A3" t="str">
-        <v>img-002</v>
-      </c>
-      <c r="B3" t="str">
-        <v>Pexels Cat</v>
-      </c>
-      <c r="C3" t="str">
-        <v>https://images.pexels.com/photos/572861/pexels-photo-572861.jpeg</v>
-      </c>
-      <c r="D3" t="str">
-        <v>2026-02-21T00:04:56.455Z</v>
-      </c>
-    </row>
-    <row r="4">
-      <c r="A4" t="str">
-        <v>img-003</v>
-      </c>
-      <c r="B4" t="str">
-        <v>Pexels Bird</v>
-      </c>
-      <c r="C4" t="str">
-        <v>https://images.pexels.com/photos/2674052/pexels-photo-2674052.jpeg</v>
-      </c>
-      <c r="D4" t="str">
-        <v>2026-02-21T00:04:56.455Z</v>
-      </c>
-    </row>
-    <row r="5">
-      <c r="A5" t="str">
-        <v>img-004</v>
-      </c>
-      <c r="B5" t="str">
-        <v>Pexels Deer</v>
-      </c>
-      <c r="C5" t="str">
-        <v>https://images.pexels.com/photos/247376/pexels-photo-247376.jpeg</v>
-      </c>
-      <c r="D5" t="str">
-        <v>2026-02-21T00:04:56.455Z</v>
-      </c>
-    </row>
-    <row r="6">
-      <c r="A6" t="str">
-        <v>img-005</v>
-      </c>
-      <c r="B6" t="str">
-        <v>Pexels Antler</v>
-      </c>
-      <c r="C6" t="str">
-        <v>https://images.pexels.com/photos/34231/antler-antler-carrier-fallow-deer-hirsch.jpg</v>
-      </c>
-      <c r="D6" t="str">
-        <v>2026-02-21T00:04:56.455Z</v>
-      </c>
-    </row>
-    <row r="7">
-      <c r="A7" t="str">
-        <v>img-006</v>
-      </c>
-      <c r="B7" t="str">
-        <v>Mountain Lake</v>
-      </c>
-      <c r="C7" t="str">
-        <v>https://images.pexels.com/photos/417173/pexels-photo-417173.jpeg</v>
-      </c>
-      <c r="D7" t="str">
-        <v>2026-02-21T00:04:56.455Z</v>
-      </c>
-    </row>
-    <row r="8">
-      <c r="A8" t="str">
-        <v>img-007</v>
-      </c>
-      <c r="B8" t="str">
-        <v>City Night</v>
-      </c>
-      <c r="C8" t="str">
-        <v>https://images.pexels.com/photos/338515/pexels-photo-338515.jpeg</v>
-      </c>
-      <c r="D8" t="str">
-        <v>2026-02-21T00:04:56.455Z</v>
-      </c>
-    </row>
-    <row r="9">
-      <c r="A9" t="str">
-        <v>img-008</v>
-      </c>
-      <c r="B9" t="str">
-        <v>Forest Trail</v>
-      </c>
-      <c r="C9" t="str">
-        <v>https://images.pexels.com/photos/4827/nature-forest-trees-fog.jpeg</v>
-      </c>
-      <c r="D9" t="str">
-        <v>2026-02-21T00:04:56.455Z</v>
-      </c>
-    </row>
-    <row r="10">
-      <c r="A10" t="str">
-        <v>img-009</v>
-      </c>
-      <c r="B10" t="str">
-        <v>Coffee Cup</v>
-      </c>
-      <c r="C10" t="str">
-        <v>https://images.pexels.com/photos/302899/pexels-photo-302899.jpeg</v>
-      </c>
-      <c r="D10" t="str">
-        <v>2026-02-21T00:04:56.455Z</v>
-      </c>
-    </row>
-    <row r="11">
-      <c r="A11" t="str">
-        <v>img-010</v>
-      </c>
-      <c r="B11" t="str">
-        <v>Laptop Desk</v>
-      </c>
-      <c r="C11" t="str">
-        <v>https://images.pexels.com/photos/18105/pexels-photo.jpg</v>
-      </c>
-      <c r="D11" t="str">
-        <v>2026-02-21T00:04:56.455Z</v>
-      </c>
-    </row>
-    <row r="12">
-      <c r="A12" t="str">
-        <v>img-011</v>
-      </c>
-      <c r="B12" t="str">
-        <v>Vintage Camera</v>
-      </c>
-      <c r="C12" t="str">
-        <v>https://images.pexels.com/photos/90946/pexels-photo-90946.jpeg</v>
-      </c>
-      <c r="D12" t="str">
-        <v>2026-02-21T00:04:56.455Z</v>
-      </c>
-    </row>
-    <row r="13">
-      <c r="A13" t="str">
-        <v>img-012</v>
-      </c>
-      <c r="B13" t="str">
-        <v>Football</v>
-      </c>
-      <c r="C13" t="str">
-        <v>https://images.pexels.com/photos/47730/the-ball-stadion-football-the-pitch-47730.jpeg</v>
-      </c>
-      <c r="D13" t="str">
-        <v>2026-02-21T00:04:56.455Z</v>
-      </c>
-    </row>
-    <row r="14">
-      <c r="A14" t="str">
-        <v>img-013</v>
-      </c>
-      <c r="B14" t="str">
-        <v>Pizza</v>
-      </c>
-      <c r="C14" t="str">
-        <v>https://images.pexels.com/photos/315755/pexels-photo-315755.jpeg</v>
-      </c>
-      <c r="D14" t="str">
-        <v>2026-02-21T00:04:56.455Z</v>
-      </c>
-    </row>
-    <row r="15">
-      <c r="A15" t="str">
-        <v>img-014</v>
-      </c>
-      <c r="B15" t="str">
-        <v>Ice Cream</v>
-      </c>
-      <c r="C15" t="str">
-        <v>https://images.pexels.com/photos/1352278/pexels-photo-1352278.jpeg</v>
-      </c>
-      <c r="D15" t="str">
-        <v>2026-02-21T00:04:56.455Z</v>
-      </c>
-    </row>
-    <row r="16">
-      <c r="A16" t="str">
-        <v>img-015</v>
-      </c>
-      <c r="B16" t="str">
-        <v>Rocket</v>
-      </c>
-      <c r="C16" t="str">
-        <v>https://images.pexels.com/photos/586063/pexels-photo-586063.jpeg</v>
-      </c>
-      <c r="D16" t="str">
-        <v>2026-02-21T00:04:56.455Z</v>
-      </c>
-    </row>
-    <row r="17">
-      <c r="A17" t="str">
-        <v>img-016</v>
-      </c>
-      <c r="B17" t="str">
-        <v>Palm Tree</v>
-      </c>
-      <c r="C17" t="str">
-        <v>https://images.pexels.com/photos/457882/pexels-photo-457882.jpeg</v>
-      </c>
-      <c r="D17" t="str">
-        <v>2026-02-21T00:04:56.455Z</v>
-      </c>
-    </row>
-    <row r="18">
-      <c r="A18" t="str">
-        <v>img-017</v>
-      </c>
-      <c r="B18" t="str">
-        <v>Castle</v>
-      </c>
-      <c r="C18" t="str">
-        <v>https://images.pexels.com/photos/161154/castle-hluboka-czech-republic-architecture-161154.jpeg</v>
-      </c>
-      <c r="D18" t="str">
-        <v>2026-02-21T00:04:56.455Z</v>
-      </c>
-    </row>
-    <row r="19">
-      <c r="A19" t="str">
-        <v>img-018</v>
-      </c>
-      <c r="B19" t="str">
-        <v>Guitar</v>
-      </c>
-      <c r="C19" t="str">
-        <v>https://images.pexels.com/photos/164938/pexels-photo-164938.jpeg</v>
-      </c>
-      <c r="D19" t="str">
-        <v>2026-02-21T00:04:56.455Z</v>
-      </c>
-    </row>
-    <row r="20">
-      <c r="A20" t="str">
-        <v>img-019</v>
-      </c>
-      <c r="B20" t="str">
-        <v>Robot</v>
-      </c>
-      <c r="C20" t="str">
-        <v>https://images.pexels.com/photos/2599244/pexels-photo-2599244.jpeg</v>
-      </c>
-      <c r="D20" t="str">
-        <v>2026-02-21T00:04:56.455Z</v>
-      </c>
-    </row>
-    <row r="21">
-      <c r="A21" t="str">
-        <v>img-020</v>
-      </c>
-      <c r="B21" t="str">
-        <v>Space</v>
-      </c>
-      <c r="C21" t="str">
-        <v>https://images.pexels.com/photos/2159/flight-sky-earth-space.jpg</v>
-      </c>
-      <c r="D21" t="str">
-        <v>2026-02-21T00:04:56.455Z</v>
-      </c>
-    </row>
-    <row r="22">
-      <c r="A22" t="str">
-        <v>img-1771632415619</v>
-      </c>
-      <c r="B22" t="str">
-        <v>omar</v>
-      </c>
-      <c r="C22" t="str">
-        <v>https://images.pexels.com/photos/667201/pexels-photo-667201.jpeg</v>
-      </c>
-      <c r="D22" t="str">
-        <v>2026-02-21T00:06:55.619Z</v>
-      </c>
-    </row>
-    <row r="23">
-      <c r="A23" t="str">
-        <v>img-1771632451515</v>
-      </c>
-      <c r="B23" t="str">
-        <v>dd</v>
-      </c>
-      <c r="C23" t="str">
-        <v>https://images.pexels.com/photos/1059823/pexels-photo-1059823.jpeg</v>
-      </c>
-      <c r="D23" t="str">
-        <v>2026-02-21T00:07:31.515Z</v>
+        <v>2026-02-21T22:16:03.648Z</v>
       </c>
     </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:D23"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:C2"/>
   </ignoredErrors>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
replace the exel file with database
</commit_message>
<xml_diff>
--- a/data/images.xlsx
+++ b/data/images.xlsx
@@ -398,17 +398,69 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1"/>
-  <sheetData/>
+  <dimension ref="A1:E3"/>
+  <sheetData>
+    <row r="1">
+      <c r="A1" t="str">
+        <v>id</v>
+      </c>
+      <c r="B1" t="str">
+        <v>label</v>
+      </c>
+      <c r="C1" t="str">
+        <v>category</v>
+      </c>
+      <c r="D1" t="str">
+        <v>url</v>
+      </c>
+      <c r="E1" t="str">
+        <v>createdAt</v>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="str">
+        <v>img-1771714971103</v>
+      </c>
+      <c r="B2" t="str">
+        <v>سعاد</v>
+      </c>
+      <c r="C2" t="str">
+        <v>باب الحارة</v>
+      </c>
+      <c r="D2" t="str">
+        <v>https://i.ytimg.com/vi/sWaza53Cs90/maxresdefault.jpg?sqp=-oaymwEmCIAKENAF8quKqQMa8AEB-AH-CYAC0AWKAgwIABABGFsgTihlMA8=&amp;rs=AOn4CLD34TVEJa_5U4E5Vf3AZBI1Hig5ZQ</v>
+      </c>
+      <c r="E2" t="str">
+        <v>2026-02-21T23:02:51.103Z</v>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="str">
+        <v>img-1771714991978</v>
+      </c>
+      <c r="B3" t="str">
+        <v>خيرية</v>
+      </c>
+      <c r="C3" t="str">
+        <v>باب الحارة</v>
+      </c>
+      <c r="D3" t="str">
+        <v>https://i1.wp.com/www.assawsana.com/portal/image/imgid399490.jpg?w=600&amp;ulb=true</v>
+      </c>
+      <c r="E3" t="str">
+        <v>2026-02-21T23:03:11.978Z</v>
+      </c>
+    </row>
+  </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:E3"/>
   </ignoredErrors>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:C2"/>
+  <dimension ref="A1:C3"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
@@ -429,12 +481,23 @@
         <v>عام</v>
       </c>
       <c r="C2" t="str">
-        <v>2026-02-21T22:16:03.648Z</v>
+        <v>2026-02-21T23:03:31.523Z</v>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="str">
+        <v>cat-002</v>
+      </c>
+      <c r="B3" t="str">
+        <v>باب الحارة</v>
+      </c>
+      <c r="C3" t="str">
+        <v>2026-02-21T23:03:31.523Z</v>
       </c>
     </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:C2"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:C3"/>
   </ignoredErrors>
 </worksheet>
 </file>
</xml_diff>